<commit_message>
#143 Add ADEE template
</commit_message>
<xml_diff>
--- a/metadata/pk_spec.xlsx
+++ b/metadata/pk_spec.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeff.dickinson\Documents\GitHub\examples\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD0C8541-8641-426F-8D37-58C16A89F5DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74A44F67-7D9A-4AE7-897D-3C4D90A5137C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Codelists!$A$1:$H$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Comments!$A$1:$D$272</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Datasets!$A$1:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Datasets!$A$1:$I$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Dictionaries!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">Documents!$A$1:$C$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Methods!$A$1:$H$1</definedName>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1618" uniqueCount="576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2342" uniqueCount="661">
   <si>
     <t>Attribute</t>
   </si>
@@ -1789,6 +1789,261 @@
   </si>
   <si>
     <t>Steady-State Cmax (ug/mL)</t>
+  </si>
+  <si>
+    <t>ADEE</t>
+  </si>
+  <si>
+    <t>Total Treatment Duration (Days)</t>
+  </si>
+  <si>
+    <t>Parameter (N)</t>
+  </si>
+  <si>
+    <t>PARCAT1</t>
+  </si>
+  <si>
+    <t>Parameter Category 1</t>
+  </si>
+  <si>
+    <t>PARCAT2</t>
+  </si>
+  <si>
+    <t>Parameter Category 2</t>
+  </si>
+  <si>
+    <t>STARTDT</t>
+  </si>
+  <si>
+    <t>Time to Event Origin Date for Subject</t>
+  </si>
+  <si>
+    <t>CNSR</t>
+  </si>
+  <si>
+    <t>Censor</t>
+  </si>
+  <si>
+    <t>EVENT</t>
+  </si>
+  <si>
+    <t>Event Indicator</t>
+  </si>
+  <si>
+    <t>EVNTDESC</t>
+  </si>
+  <si>
+    <t>Event or Censoring Description</t>
+  </si>
+  <si>
+    <t>Source Data</t>
+  </si>
+  <si>
+    <t>Source Sequence Number</t>
+  </si>
+  <si>
+    <t>ANL03FL</t>
+  </si>
+  <si>
+    <t>Analysis Flag 03</t>
+  </si>
+  <si>
+    <t>ANL04FL</t>
+  </si>
+  <si>
+    <t>Analysis Flag 04</t>
+  </si>
+  <si>
+    <t>ADES</t>
+  </si>
+  <si>
+    <t>Planned Arm Code (N)</t>
+  </si>
+  <si>
+    <t>TRT01PN</t>
+  </si>
+  <si>
+    <t>Planned Treatment for Period 01 (N)</t>
+  </si>
+  <si>
+    <t>TRT01AN</t>
+  </si>
+  <si>
+    <t>Actual Treatment for Period 01 (N)</t>
+  </si>
+  <si>
+    <t>AVALC</t>
+  </si>
+  <si>
+    <t>Analysis Value (C)</t>
+  </si>
+  <si>
+    <t>AESEQ</t>
+  </si>
+  <si>
+    <t>Adverse Event Sequence Number</t>
+  </si>
+  <si>
+    <t>AESPID</t>
+  </si>
+  <si>
+    <t>Sponsor-Defined Identifier</t>
+  </si>
+  <si>
+    <t>AEDECOD</t>
+  </si>
+  <si>
+    <t>Dictionary-Derived Term</t>
+  </si>
+  <si>
+    <t>AEBODSYS</t>
+  </si>
+  <si>
+    <t>Body System or Organ Class</t>
+  </si>
+  <si>
+    <t>ASEV</t>
+  </si>
+  <si>
+    <t>Severity (MILD/MODERATE/SEVERE)</t>
+  </si>
+  <si>
+    <t>ASEVN</t>
+  </si>
+  <si>
+    <t>Severity (N) (1/2/3)</t>
+  </si>
+  <si>
+    <t>AEREL</t>
+  </si>
+  <si>
+    <t>Causality</t>
+  </si>
+  <si>
+    <t>AERELN</t>
+  </si>
+  <si>
+    <t>Causality (N) (0-4)</t>
+  </si>
+  <si>
+    <t>AESER</t>
+  </si>
+  <si>
+    <t>Serious Event</t>
+  </si>
+  <si>
+    <t>AEACN</t>
+  </si>
+  <si>
+    <t>Action Taken with Study Treatment</t>
+  </si>
+  <si>
+    <t>AEOUT</t>
+  </si>
+  <si>
+    <t>Outcome of Adverse Event</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>ASTDY</t>
+  </si>
+  <si>
+    <t>Analysis Start Relative Day</t>
+  </si>
+  <si>
+    <t>AENDY</t>
+  </si>
+  <si>
+    <t>Analysis End Relative Day</t>
+  </si>
+  <si>
+    <t>ADURN</t>
+  </si>
+  <si>
+    <t>Analysis Duration</t>
+  </si>
+  <si>
+    <t>ADURU</t>
+  </si>
+  <si>
+    <t>Analysis Duration Units</t>
+  </si>
+  <si>
+    <t>TRTEMFL</t>
+  </si>
+  <si>
+    <t>Treatment Emergent Analysis Flag</t>
+  </si>
+  <si>
+    <t>Steady-State Area Under Curve</t>
+  </si>
+  <si>
+    <t>Steady-State Maximum Concentration</t>
+  </si>
+  <si>
+    <t>Baseline Body Mass Index (kg/m2)</t>
+  </si>
+  <si>
+    <t>Baseline Body Surface Area (m2)</t>
+  </si>
+  <si>
+    <t>Baseline Creatinine (mg/dL)</t>
+  </si>
+  <si>
+    <t>Baseline eGFR (mL/min/1.73m2)</t>
+  </si>
+  <si>
+    <t>Analysis Flag 01 (Primary Analysis)</t>
+  </si>
+  <si>
+    <t>Analysis Flag 02 (Event-Level Analysis)</t>
+  </si>
+  <si>
+    <t>ADTRR</t>
+  </si>
+  <si>
+    <t>PCHG</t>
+  </si>
+  <si>
+    <t>Percent Change from Baseline</t>
+  </si>
+  <si>
+    <t>NADIR</t>
+  </si>
+  <si>
+    <t>Nadir Value</t>
+  </si>
+  <si>
+    <t>NADPCHG</t>
+  </si>
+  <si>
+    <t>Percent Change from Nadir</t>
+  </si>
+  <si>
+    <t>BORN</t>
+  </si>
+  <si>
+    <t>Best Overall Response (N)</t>
+  </si>
+  <si>
+    <t>Analysis Flag 02 (Post-Baseline Records)</t>
+  </si>
+  <si>
+    <t>Analysis Flag 03 (Confirmed Response)</t>
+  </si>
+  <si>
+    <t>Exposure Efficacy Analysis Data</t>
+  </si>
+  <si>
+    <t>STUDYID, USUBJID, PARAMCD</t>
+  </si>
+  <si>
+    <t>Exposure Safety Analysis Data</t>
+  </si>
+  <si>
+    <t>Exposure Tumor Response</t>
   </si>
 </sst>
 </file>
@@ -1878,7 +2133,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
@@ -1957,6 +2212,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -2395,7 +2653,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" style="15" customWidth="1"/>
@@ -2517,38 +2775,89 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="12"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="12"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="12"/>
+    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="29" t="s">
+        <v>576</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>657</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>392</v>
+      </c>
+      <c r="D5" s="29"/>
+      <c r="E5" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>658</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>393</v>
+      </c>
+      <c r="H5"/>
+      <c r="I5" s="17" t="s">
+        <v>394</v>
+      </c>
+      <c r="J5" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="29" t="s">
+        <v>597</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>659</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>392</v>
+      </c>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="29" t="s">
+        <v>658</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>393</v>
+      </c>
+      <c r="H6"/>
+      <c r="I6" s="17" t="s">
+        <v>394</v>
+      </c>
+      <c r="J6" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="29" t="s">
+        <v>646</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>660</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>392</v>
+      </c>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="29" t="s">
+        <v>658</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>393</v>
+      </c>
+      <c r="H7"/>
+      <c r="I7" s="17" t="s">
+        <v>394</v>
+      </c>
+      <c r="J7" s="14" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
@@ -2561,19 +2870,8 @@
       <c r="H8" s="11"/>
       <c r="I8" s="12"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="12"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I9" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:I8" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K737373 Public</oddFooter>
@@ -2583,7 +2881,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P259"/>
+  <dimension ref="A1:P411"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" style="28" customWidth="1"/>
@@ -8119,70 +8417,3245 @@
       </c>
     </row>
     <row r="238" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A238"/>
+      <c r="A238">
+        <v>48</v>
+      </c>
+      <c r="B238" t="s">
+        <v>576</v>
+      </c>
+      <c r="C238" t="s">
+        <v>51</v>
+      </c>
+      <c r="D238" t="s">
+        <v>82</v>
+      </c>
+      <c r="E238" t="s">
+        <v>108</v>
+      </c>
+      <c r="F238">
+        <v>20</v>
+      </c>
     </row>
     <row r="239" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A239"/>
+      <c r="A239">
+        <v>49</v>
+      </c>
+      <c r="B239" t="s">
+        <v>576</v>
+      </c>
+      <c r="C239" t="s">
+        <v>52</v>
+      </c>
+      <c r="D239" t="s">
+        <v>83</v>
+      </c>
+      <c r="E239" t="s">
+        <v>108</v>
+      </c>
+      <c r="F239">
+        <v>40</v>
+      </c>
     </row>
     <row r="240" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A240"/>
-    </row>
-    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A241"/>
-    </row>
-    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A242"/>
-    </row>
-    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A243"/>
-    </row>
-    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A244"/>
-    </row>
-    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A245"/>
-    </row>
-    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A246"/>
-    </row>
-    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A247"/>
-    </row>
-    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A248"/>
-    </row>
-    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A249" s="27"/>
-    </row>
-    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A250" s="27"/>
-    </row>
-    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A251" s="27"/>
-    </row>
-    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A252" s="27"/>
-    </row>
-    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A253" s="27"/>
-    </row>
-    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A254" s="27"/>
-    </row>
-    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A255" s="27"/>
-    </row>
-    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A256" s="27"/>
-    </row>
-    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A257" s="27"/>
-    </row>
-    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A258" s="27"/>
-    </row>
-    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A259" s="27"/>
+      <c r="A240">
+        <v>50</v>
+      </c>
+      <c r="B240" t="s">
+        <v>576</v>
+      </c>
+      <c r="C240" t="s">
+        <v>55</v>
+      </c>
+      <c r="D240" t="s">
+        <v>89</v>
+      </c>
+      <c r="E240" t="s">
+        <v>108</v>
+      </c>
+      <c r="F240">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="241" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A241">
+        <v>51</v>
+      </c>
+      <c r="B241" t="s">
+        <v>576</v>
+      </c>
+      <c r="C241" t="s">
+        <v>64</v>
+      </c>
+      <c r="D241" t="s">
+        <v>97</v>
+      </c>
+      <c r="E241" t="s">
+        <v>108</v>
+      </c>
+      <c r="F241">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="242" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A242">
+        <v>52</v>
+      </c>
+      <c r="B242" t="s">
+        <v>576</v>
+      </c>
+      <c r="C242" t="s">
+        <v>65</v>
+      </c>
+      <c r="D242" t="s">
+        <v>98</v>
+      </c>
+      <c r="E242" t="s">
+        <v>528</v>
+      </c>
+      <c r="F242">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="243" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A243">
+        <v>55</v>
+      </c>
+      <c r="B243" t="s">
+        <v>576</v>
+      </c>
+      <c r="C243" t="s">
+        <v>67</v>
+      </c>
+      <c r="D243" t="s">
+        <v>100</v>
+      </c>
+      <c r="E243" t="s">
+        <v>108</v>
+      </c>
+      <c r="F243">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A244">
+        <v>56</v>
+      </c>
+      <c r="B244" t="s">
+        <v>576</v>
+      </c>
+      <c r="C244" t="s">
+        <v>480</v>
+      </c>
+      <c r="D244" t="s">
+        <v>481</v>
+      </c>
+      <c r="E244" t="s">
+        <v>528</v>
+      </c>
+      <c r="F244">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="245" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A245">
+        <v>57</v>
+      </c>
+      <c r="B245" t="s">
+        <v>576</v>
+      </c>
+      <c r="C245" t="s">
+        <v>68</v>
+      </c>
+      <c r="D245" t="s">
+        <v>101</v>
+      </c>
+      <c r="E245" t="s">
+        <v>108</v>
+      </c>
+      <c r="F245">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="246" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A246">
+        <v>58</v>
+      </c>
+      <c r="B246" t="s">
+        <v>576</v>
+      </c>
+      <c r="C246" t="s">
+        <v>482</v>
+      </c>
+      <c r="D246" t="s">
+        <v>483</v>
+      </c>
+      <c r="E246" t="s">
+        <v>528</v>
+      </c>
+      <c r="F246">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="247" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A247">
+        <v>12</v>
+      </c>
+      <c r="B247" t="s">
+        <v>576</v>
+      </c>
+      <c r="C247" t="s">
+        <v>69</v>
+      </c>
+      <c r="D247" t="s">
+        <v>531</v>
+      </c>
+      <c r="E247" t="s">
+        <v>108</v>
+      </c>
+      <c r="F247">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="248" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A248">
+        <v>13</v>
+      </c>
+      <c r="B248" t="s">
+        <v>576</v>
+      </c>
+      <c r="C248" t="s">
+        <v>71</v>
+      </c>
+      <c r="D248" t="s">
+        <v>103</v>
+      </c>
+      <c r="E248" t="s">
+        <v>108</v>
+      </c>
+      <c r="F248">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="249" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A249">
+        <v>14</v>
+      </c>
+      <c r="B249" t="s">
+        <v>576</v>
+      </c>
+      <c r="C249" t="s">
+        <v>518</v>
+      </c>
+      <c r="D249" t="s">
+        <v>536</v>
+      </c>
+      <c r="E249" t="s">
+        <v>528</v>
+      </c>
+      <c r="F249">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="250" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A250">
+        <v>15</v>
+      </c>
+      <c r="B250" t="s">
+        <v>576</v>
+      </c>
+      <c r="C250" t="s">
+        <v>73</v>
+      </c>
+      <c r="D250" t="s">
+        <v>105</v>
+      </c>
+      <c r="E250" t="s">
+        <v>108</v>
+      </c>
+      <c r="F250">
+        <v>40</v>
+      </c>
+      <c r="H250" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="251" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A251">
+        <v>16</v>
+      </c>
+      <c r="B251" t="s">
+        <v>576</v>
+      </c>
+      <c r="C251" t="s">
+        <v>537</v>
+      </c>
+      <c r="D251" t="s">
+        <v>538</v>
+      </c>
+      <c r="E251" t="s">
+        <v>528</v>
+      </c>
+      <c r="F251">
+        <v>8</v>
+      </c>
+      <c r="H251" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="252" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A252">
+        <v>17</v>
+      </c>
+      <c r="B252" t="s">
+        <v>576</v>
+      </c>
+      <c r="C252" t="s">
+        <v>219</v>
+      </c>
+      <c r="D252" t="s">
+        <v>220</v>
+      </c>
+      <c r="E252" t="s">
+        <v>528</v>
+      </c>
+      <c r="F252">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="253" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A253">
+        <v>18</v>
+      </c>
+      <c r="B253" t="s">
+        <v>576</v>
+      </c>
+      <c r="C253" t="s">
+        <v>221</v>
+      </c>
+      <c r="D253" t="s">
+        <v>222</v>
+      </c>
+      <c r="E253" t="s">
+        <v>528</v>
+      </c>
+      <c r="F253">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="254" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A254">
+        <v>19</v>
+      </c>
+      <c r="B254" t="s">
+        <v>576</v>
+      </c>
+      <c r="C254" t="s">
+        <v>230</v>
+      </c>
+      <c r="D254" t="s">
+        <v>577</v>
+      </c>
+      <c r="E254" t="s">
+        <v>528</v>
+      </c>
+      <c r="F254">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="255" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A255">
+        <v>20</v>
+      </c>
+      <c r="B255" t="s">
+        <v>576</v>
+      </c>
+      <c r="C255" t="s">
+        <v>256</v>
+      </c>
+      <c r="D255" t="s">
+        <v>257</v>
+      </c>
+      <c r="E255" t="s">
+        <v>108</v>
+      </c>
+      <c r="F255">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="256" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A256">
+        <v>21</v>
+      </c>
+      <c r="B256" t="s">
+        <v>576</v>
+      </c>
+      <c r="C256" t="s">
+        <v>252</v>
+      </c>
+      <c r="D256" t="s">
+        <v>253</v>
+      </c>
+      <c r="E256" t="s">
+        <v>108</v>
+      </c>
+      <c r="F256">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="257" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A257">
+        <v>22</v>
+      </c>
+      <c r="B257" t="s">
+        <v>576</v>
+      </c>
+      <c r="C257" t="s">
+        <v>254</v>
+      </c>
+      <c r="D257" t="s">
+        <v>578</v>
+      </c>
+      <c r="E257" t="s">
+        <v>528</v>
+      </c>
+      <c r="F257">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="258" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A258">
+        <v>23</v>
+      </c>
+      <c r="B258" t="s">
+        <v>576</v>
+      </c>
+      <c r="C258" t="s">
+        <v>579</v>
+      </c>
+      <c r="D258" t="s">
+        <v>580</v>
+      </c>
+      <c r="E258" t="s">
+        <v>108</v>
+      </c>
+      <c r="F258">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="259" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A259">
+        <v>24</v>
+      </c>
+      <c r="B259" t="s">
+        <v>576</v>
+      </c>
+      <c r="C259" t="s">
+        <v>581</v>
+      </c>
+      <c r="D259" t="s">
+        <v>582</v>
+      </c>
+      <c r="E259" t="s">
+        <v>108</v>
+      </c>
+      <c r="F259">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="260" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A260">
+        <v>25</v>
+      </c>
+      <c r="B260" t="s">
+        <v>576</v>
+      </c>
+      <c r="C260" t="s">
+        <v>312</v>
+      </c>
+      <c r="D260" t="s">
+        <v>313</v>
+      </c>
+      <c r="E260" t="s">
+        <v>544</v>
+      </c>
+      <c r="F260">
+        <v>8</v>
+      </c>
+      <c r="H260" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="261" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A261">
+        <v>26</v>
+      </c>
+      <c r="B261" t="s">
+        <v>576</v>
+      </c>
+      <c r="C261" t="s">
+        <v>314</v>
+      </c>
+      <c r="D261" t="s">
+        <v>315</v>
+      </c>
+      <c r="E261" t="s">
+        <v>108</v>
+      </c>
+      <c r="F261">
+        <v>20</v>
+      </c>
+      <c r="H261" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="262" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A262">
+        <v>28</v>
+      </c>
+      <c r="B262" t="s">
+        <v>576</v>
+      </c>
+      <c r="C262" t="s">
+        <v>300</v>
+      </c>
+      <c r="D262" t="s">
+        <v>301</v>
+      </c>
+      <c r="E262" t="s">
+        <v>528</v>
+      </c>
+      <c r="F262">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="263" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A263">
+        <v>29</v>
+      </c>
+      <c r="B263" t="s">
+        <v>576</v>
+      </c>
+      <c r="C263" t="s">
+        <v>583</v>
+      </c>
+      <c r="D263" t="s">
+        <v>584</v>
+      </c>
+      <c r="E263" t="s">
+        <v>528</v>
+      </c>
+      <c r="F263">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="264" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A264">
+        <v>30</v>
+      </c>
+      <c r="B264" t="s">
+        <v>576</v>
+      </c>
+      <c r="C264" t="s">
+        <v>585</v>
+      </c>
+      <c r="D264" t="s">
+        <v>586</v>
+      </c>
+      <c r="E264" t="s">
+        <v>528</v>
+      </c>
+      <c r="F264">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="265" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A265">
+        <v>31</v>
+      </c>
+      <c r="B265" t="s">
+        <v>576</v>
+      </c>
+      <c r="C265" t="s">
+        <v>587</v>
+      </c>
+      <c r="D265" t="s">
+        <v>588</v>
+      </c>
+      <c r="E265" t="s">
+        <v>528</v>
+      </c>
+      <c r="F265">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="266" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A266">
+        <v>32</v>
+      </c>
+      <c r="B266" t="s">
+        <v>576</v>
+      </c>
+      <c r="C266" t="s">
+        <v>589</v>
+      </c>
+      <c r="D266" t="s">
+        <v>590</v>
+      </c>
+      <c r="E266" t="s">
+        <v>108</v>
+      </c>
+      <c r="F266">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="267" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A267">
+        <v>33</v>
+      </c>
+      <c r="B267" t="s">
+        <v>576</v>
+      </c>
+      <c r="C267" t="s">
+        <v>386</v>
+      </c>
+      <c r="D267" t="s">
+        <v>591</v>
+      </c>
+      <c r="E267" t="s">
+        <v>108</v>
+      </c>
+      <c r="F267">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="268" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A268">
+        <v>34</v>
+      </c>
+      <c r="B268" t="s">
+        <v>576</v>
+      </c>
+      <c r="C268" t="s">
+        <v>388</v>
+      </c>
+      <c r="D268" t="s">
+        <v>389</v>
+      </c>
+      <c r="E268" t="s">
+        <v>108</v>
+      </c>
+      <c r="F268">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="269" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A269">
+        <v>35</v>
+      </c>
+      <c r="B269" t="s">
+        <v>576</v>
+      </c>
+      <c r="C269" t="s">
+        <v>390</v>
+      </c>
+      <c r="D269" t="s">
+        <v>592</v>
+      </c>
+      <c r="E269" t="s">
+        <v>528</v>
+      </c>
+      <c r="F269">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="270" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A270">
+        <v>40</v>
+      </c>
+      <c r="B270" t="s">
+        <v>576</v>
+      </c>
+      <c r="C270" t="s">
+        <v>572</v>
+      </c>
+      <c r="D270" t="s">
+        <v>573</v>
+      </c>
+      <c r="E270" t="s">
+        <v>544</v>
+      </c>
+      <c r="F270">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="271" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A271">
+        <v>49</v>
+      </c>
+      <c r="B271" t="s">
+        <v>576</v>
+      </c>
+      <c r="C271" t="s">
+        <v>574</v>
+      </c>
+      <c r="D271" t="s">
+        <v>575</v>
+      </c>
+      <c r="E271" t="s">
+        <v>544</v>
+      </c>
+      <c r="F271">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="272" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A272">
+        <v>52</v>
+      </c>
+      <c r="B272" t="s">
+        <v>576</v>
+      </c>
+      <c r="C272" t="s">
+        <v>372</v>
+      </c>
+      <c r="D272" t="s">
+        <v>560</v>
+      </c>
+      <c r="E272" t="s">
+        <v>544</v>
+      </c>
+      <c r="F272">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A273">
+        <v>54</v>
+      </c>
+      <c r="B273" t="s">
+        <v>576</v>
+      </c>
+      <c r="C273" t="s">
+        <v>374</v>
+      </c>
+      <c r="D273" t="s">
+        <v>561</v>
+      </c>
+      <c r="E273" t="s">
+        <v>544</v>
+      </c>
+      <c r="F273">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A274">
+        <v>55</v>
+      </c>
+      <c r="B274" t="s">
+        <v>576</v>
+      </c>
+      <c r="C274" t="s">
+        <v>376</v>
+      </c>
+      <c r="D274" t="s">
+        <v>562</v>
+      </c>
+      <c r="E274" t="s">
+        <v>544</v>
+      </c>
+      <c r="F274">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="275" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A275">
+        <v>56</v>
+      </c>
+      <c r="B275" t="s">
+        <v>576</v>
+      </c>
+      <c r="C275" t="s">
+        <v>477</v>
+      </c>
+      <c r="D275" t="s">
+        <v>563</v>
+      </c>
+      <c r="E275" t="s">
+        <v>544</v>
+      </c>
+      <c r="F275">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A276">
+        <v>57</v>
+      </c>
+      <c r="B276" t="s">
+        <v>576</v>
+      </c>
+      <c r="C276" t="s">
+        <v>494</v>
+      </c>
+      <c r="D276" t="s">
+        <v>564</v>
+      </c>
+      <c r="E276" t="s">
+        <v>544</v>
+      </c>
+      <c r="F276">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="277" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A277">
+        <v>58</v>
+      </c>
+      <c r="B277" t="s">
+        <v>576</v>
+      </c>
+      <c r="C277" t="s">
+        <v>496</v>
+      </c>
+      <c r="D277" t="s">
+        <v>565</v>
+      </c>
+      <c r="E277" t="s">
+        <v>544</v>
+      </c>
+      <c r="F277">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A278">
+        <v>59</v>
+      </c>
+      <c r="B278" t="s">
+        <v>576</v>
+      </c>
+      <c r="C278" t="s">
+        <v>498</v>
+      </c>
+      <c r="D278" t="s">
+        <v>566</v>
+      </c>
+      <c r="E278" t="s">
+        <v>544</v>
+      </c>
+      <c r="F278">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A279">
+        <v>60</v>
+      </c>
+      <c r="B279" t="s">
+        <v>576</v>
+      </c>
+      <c r="C279" t="s">
+        <v>504</v>
+      </c>
+      <c r="D279" t="s">
+        <v>567</v>
+      </c>
+      <c r="E279" t="s">
+        <v>544</v>
+      </c>
+      <c r="F279">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A280">
+        <v>61</v>
+      </c>
+      <c r="B280" t="s">
+        <v>576</v>
+      </c>
+      <c r="C280" t="s">
+        <v>502</v>
+      </c>
+      <c r="D280" t="s">
+        <v>568</v>
+      </c>
+      <c r="E280" t="s">
+        <v>544</v>
+      </c>
+      <c r="F280">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A281">
+        <v>62</v>
+      </c>
+      <c r="B281" t="s">
+        <v>576</v>
+      </c>
+      <c r="C281" t="s">
+        <v>500</v>
+      </c>
+      <c r="D281" t="s">
+        <v>569</v>
+      </c>
+      <c r="E281" t="s">
+        <v>544</v>
+      </c>
+      <c r="F281">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="282" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A282">
+        <v>64</v>
+      </c>
+      <c r="B282" t="s">
+        <v>576</v>
+      </c>
+      <c r="C282" t="s">
+        <v>328</v>
+      </c>
+      <c r="D282" t="s">
+        <v>329</v>
+      </c>
+      <c r="E282" t="s">
+        <v>108</v>
+      </c>
+      <c r="F282">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="283" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A283">
+        <v>65</v>
+      </c>
+      <c r="B283" t="s">
+        <v>576</v>
+      </c>
+      <c r="C283" t="s">
+        <v>326</v>
+      </c>
+      <c r="D283" t="s">
+        <v>327</v>
+      </c>
+      <c r="E283" t="s">
+        <v>108</v>
+      </c>
+      <c r="F283">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A284">
+        <v>66</v>
+      </c>
+      <c r="B284" t="s">
+        <v>576</v>
+      </c>
+      <c r="C284" t="s">
+        <v>593</v>
+      </c>
+      <c r="D284" t="s">
+        <v>594</v>
+      </c>
+      <c r="E284" t="s">
+        <v>108</v>
+      </c>
+      <c r="F284">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="285" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A285">
+        <v>67</v>
+      </c>
+      <c r="B285" t="s">
+        <v>576</v>
+      </c>
+      <c r="C285" t="s">
+        <v>595</v>
+      </c>
+      <c r="D285" t="s">
+        <v>596</v>
+      </c>
+      <c r="E285" t="s">
+        <v>108</v>
+      </c>
+      <c r="F285">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="286" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A286">
+        <v>68</v>
+      </c>
+      <c r="B286" t="s">
+        <v>576</v>
+      </c>
+      <c r="C286" t="s">
+        <v>384</v>
+      </c>
+      <c r="D286" t="s">
+        <v>385</v>
+      </c>
+      <c r="E286" t="s">
+        <v>528</v>
+      </c>
+      <c r="F286">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="287" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A287">
+        <v>1</v>
+      </c>
+      <c r="B287" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C287" t="s">
+        <v>51</v>
+      </c>
+      <c r="D287" t="s">
+        <v>82</v>
+      </c>
+      <c r="E287" t="s">
+        <v>108</v>
+      </c>
+      <c r="F287">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="288" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A288">
+        <v>2</v>
+      </c>
+      <c r="B288" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C288" t="s">
+        <v>402</v>
+      </c>
+      <c r="D288" t="s">
+        <v>403</v>
+      </c>
+      <c r="E288" t="s">
+        <v>528</v>
+      </c>
+      <c r="F288"/>
+    </row>
+    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A289">
+        <v>3</v>
+      </c>
+      <c r="B289" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C289" t="s">
+        <v>52</v>
+      </c>
+      <c r="D289" t="s">
+        <v>83</v>
+      </c>
+      <c r="E289" t="s">
+        <v>108</v>
+      </c>
+      <c r="F289">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A290">
+        <v>4</v>
+      </c>
+      <c r="B290" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C290" t="s">
+        <v>411</v>
+      </c>
+      <c r="D290" t="s">
+        <v>412</v>
+      </c>
+      <c r="E290" t="s">
+        <v>528</v>
+      </c>
+      <c r="F290"/>
+    </row>
+    <row r="291" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A291">
+        <v>5</v>
+      </c>
+      <c r="B291" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C291" t="s">
+        <v>55</v>
+      </c>
+      <c r="D291" t="s">
+        <v>89</v>
+      </c>
+      <c r="E291" t="s">
+        <v>108</v>
+      </c>
+      <c r="F291">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="292" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A292">
+        <v>6</v>
+      </c>
+      <c r="B292" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C292" t="s">
+        <v>413</v>
+      </c>
+      <c r="D292" t="s">
+        <v>414</v>
+      </c>
+      <c r="E292" t="s">
+        <v>528</v>
+      </c>
+      <c r="F292"/>
+    </row>
+    <row r="293" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A293">
+        <v>7</v>
+      </c>
+      <c r="B293" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C293" t="s">
+        <v>64</v>
+      </c>
+      <c r="D293" t="s">
+        <v>97</v>
+      </c>
+      <c r="E293" t="s">
+        <v>108</v>
+      </c>
+      <c r="F293">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A294">
+        <v>8</v>
+      </c>
+      <c r="B294" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C294" t="s">
+        <v>415</v>
+      </c>
+      <c r="D294" t="s">
+        <v>416</v>
+      </c>
+      <c r="E294" t="s">
+        <v>528</v>
+      </c>
+      <c r="F294"/>
+    </row>
+    <row r="295" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A295">
+        <v>9</v>
+      </c>
+      <c r="B295" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C295" t="s">
+        <v>384</v>
+      </c>
+      <c r="D295" t="s">
+        <v>385</v>
+      </c>
+      <c r="E295" t="s">
+        <v>528</v>
+      </c>
+      <c r="F295"/>
+    </row>
+    <row r="296" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A296">
+        <v>10</v>
+      </c>
+      <c r="B296" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C296" t="s">
+        <v>71</v>
+      </c>
+      <c r="D296" t="s">
+        <v>103</v>
+      </c>
+      <c r="E296" t="s">
+        <v>108</v>
+      </c>
+      <c r="F296">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="297" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A297">
+        <v>11</v>
+      </c>
+      <c r="B297" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C297" t="s">
+        <v>518</v>
+      </c>
+      <c r="D297" t="s">
+        <v>598</v>
+      </c>
+      <c r="E297" t="s">
+        <v>528</v>
+      </c>
+      <c r="F297"/>
+    </row>
+    <row r="298" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A298">
+        <v>12</v>
+      </c>
+      <c r="B298" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C298" t="s">
+        <v>70</v>
+      </c>
+      <c r="D298" t="s">
+        <v>102</v>
+      </c>
+      <c r="E298" t="s">
+        <v>108</v>
+      </c>
+      <c r="F298">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="299" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A299">
+        <v>13</v>
+      </c>
+      <c r="B299" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C299" t="s">
+        <v>206</v>
+      </c>
+      <c r="D299" t="s">
+        <v>207</v>
+      </c>
+      <c r="E299" t="s">
+        <v>108</v>
+      </c>
+      <c r="F299">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A300">
+        <v>14</v>
+      </c>
+      <c r="B300" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C300" t="s">
+        <v>599</v>
+      </c>
+      <c r="D300" t="s">
+        <v>600</v>
+      </c>
+      <c r="E300" t="s">
+        <v>528</v>
+      </c>
+      <c r="F300"/>
+    </row>
+    <row r="301" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A301">
+        <v>15</v>
+      </c>
+      <c r="B301" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C301" t="s">
+        <v>208</v>
+      </c>
+      <c r="D301" t="s">
+        <v>209</v>
+      </c>
+      <c r="E301" t="s">
+        <v>108</v>
+      </c>
+      <c r="F301">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="302" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A302">
+        <v>16</v>
+      </c>
+      <c r="B302" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C302" t="s">
+        <v>601</v>
+      </c>
+      <c r="D302" t="s">
+        <v>602</v>
+      </c>
+      <c r="E302" t="s">
+        <v>528</v>
+      </c>
+      <c r="F302"/>
+    </row>
+    <row r="303" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A303">
+        <v>18</v>
+      </c>
+      <c r="B303" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C303" t="s">
+        <v>65</v>
+      </c>
+      <c r="D303" t="s">
+        <v>98</v>
+      </c>
+      <c r="E303" t="s">
+        <v>528</v>
+      </c>
+      <c r="F303"/>
+    </row>
+    <row r="304" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A304">
+        <v>21</v>
+      </c>
+      <c r="B304" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C304" t="s">
+        <v>67</v>
+      </c>
+      <c r="D304" t="s">
+        <v>100</v>
+      </c>
+      <c r="E304" t="s">
+        <v>108</v>
+      </c>
+      <c r="F304">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="305" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A305">
+        <v>22</v>
+      </c>
+      <c r="B305" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C305" t="s">
+        <v>480</v>
+      </c>
+      <c r="D305" t="s">
+        <v>481</v>
+      </c>
+      <c r="E305" t="s">
+        <v>528</v>
+      </c>
+      <c r="F305"/>
+    </row>
+    <row r="306" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A306">
+        <v>23</v>
+      </c>
+      <c r="B306" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C306" t="s">
+        <v>68</v>
+      </c>
+      <c r="D306" t="s">
+        <v>101</v>
+      </c>
+      <c r="E306" t="s">
+        <v>108</v>
+      </c>
+      <c r="F306">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="307" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A307">
+        <v>24</v>
+      </c>
+      <c r="B307" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C307" t="s">
+        <v>482</v>
+      </c>
+      <c r="D307" t="s">
+        <v>483</v>
+      </c>
+      <c r="E307" t="s">
+        <v>528</v>
+      </c>
+      <c r="F307"/>
+    </row>
+    <row r="308" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A308">
+        <v>25</v>
+      </c>
+      <c r="B308" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C308" t="s">
+        <v>69</v>
+      </c>
+      <c r="D308" t="s">
+        <v>531</v>
+      </c>
+      <c r="E308" t="s">
+        <v>108</v>
+      </c>
+      <c r="F308">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="309" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A309">
+        <v>26</v>
+      </c>
+      <c r="B309" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C309" t="s">
+        <v>532</v>
+      </c>
+      <c r="D309" t="s">
+        <v>533</v>
+      </c>
+      <c r="E309" t="s">
+        <v>528</v>
+      </c>
+      <c r="F309"/>
+    </row>
+    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A310">
+        <v>27</v>
+      </c>
+      <c r="B310" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C310" t="s">
+        <v>256</v>
+      </c>
+      <c r="D310" t="s">
+        <v>257</v>
+      </c>
+      <c r="E310" t="s">
+        <v>108</v>
+      </c>
+      <c r="F310">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="311" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A311">
+        <v>28</v>
+      </c>
+      <c r="B311" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C311" t="s">
+        <v>252</v>
+      </c>
+      <c r="D311" t="s">
+        <v>253</v>
+      </c>
+      <c r="E311" t="s">
+        <v>108</v>
+      </c>
+      <c r="F311">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="312" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A312">
+        <v>29</v>
+      </c>
+      <c r="B312" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C312" t="s">
+        <v>254</v>
+      </c>
+      <c r="D312" t="s">
+        <v>578</v>
+      </c>
+      <c r="E312" t="s">
+        <v>528</v>
+      </c>
+      <c r="F312"/>
+    </row>
+    <row r="313" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A313">
+        <v>30</v>
+      </c>
+      <c r="B313" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C313" t="s">
+        <v>312</v>
+      </c>
+      <c r="D313" t="s">
+        <v>313</v>
+      </c>
+      <c r="E313" t="s">
+        <v>544</v>
+      </c>
+      <c r="F313"/>
+    </row>
+    <row r="314" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A314">
+        <v>31</v>
+      </c>
+      <c r="B314" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C314" t="s">
+        <v>603</v>
+      </c>
+      <c r="D314" t="s">
+        <v>604</v>
+      </c>
+      <c r="E314" t="s">
+        <v>108</v>
+      </c>
+      <c r="F314">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="315" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A315">
+        <v>32</v>
+      </c>
+      <c r="B315" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C315" t="s">
+        <v>605</v>
+      </c>
+      <c r="D315" t="s">
+        <v>606</v>
+      </c>
+      <c r="E315" t="s">
+        <v>528</v>
+      </c>
+      <c r="F315"/>
+    </row>
+    <row r="316" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A316">
+        <v>33</v>
+      </c>
+      <c r="B316" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C316" t="s">
+        <v>607</v>
+      </c>
+      <c r="D316" t="s">
+        <v>608</v>
+      </c>
+      <c r="E316" t="s">
+        <v>108</v>
+      </c>
+      <c r="F316">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="317" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A317">
+        <v>34</v>
+      </c>
+      <c r="B317" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C317" t="s">
+        <v>609</v>
+      </c>
+      <c r="D317" t="s">
+        <v>610</v>
+      </c>
+      <c r="E317" t="s">
+        <v>108</v>
+      </c>
+      <c r="F317">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="318" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A318">
+        <v>35</v>
+      </c>
+      <c r="B318" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C318" t="s">
+        <v>611</v>
+      </c>
+      <c r="D318" t="s">
+        <v>612</v>
+      </c>
+      <c r="E318" t="s">
+        <v>108</v>
+      </c>
+      <c r="F318">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="319" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A319">
+        <v>36</v>
+      </c>
+      <c r="B319" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C319" t="s">
+        <v>613</v>
+      </c>
+      <c r="D319" t="s">
+        <v>614</v>
+      </c>
+      <c r="E319" t="s">
+        <v>108</v>
+      </c>
+      <c r="F319">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="320" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A320">
+        <v>37</v>
+      </c>
+      <c r="B320" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C320" t="s">
+        <v>615</v>
+      </c>
+      <c r="D320" t="s">
+        <v>616</v>
+      </c>
+      <c r="E320" t="s">
+        <v>528</v>
+      </c>
+      <c r="F320"/>
+    </row>
+    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A321">
+        <v>38</v>
+      </c>
+      <c r="B321" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C321" t="s">
+        <v>617</v>
+      </c>
+      <c r="D321" t="s">
+        <v>618</v>
+      </c>
+      <c r="E321" t="s">
+        <v>108</v>
+      </c>
+      <c r="F321">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="322" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A322">
+        <v>39</v>
+      </c>
+      <c r="B322" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C322" t="s">
+        <v>619</v>
+      </c>
+      <c r="D322" t="s">
+        <v>620</v>
+      </c>
+      <c r="E322" t="s">
+        <v>528</v>
+      </c>
+      <c r="F322"/>
+    </row>
+    <row r="323" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A323">
+        <v>40</v>
+      </c>
+      <c r="B323" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C323" t="s">
+        <v>621</v>
+      </c>
+      <c r="D323" t="s">
+        <v>622</v>
+      </c>
+      <c r="E323" t="s">
+        <v>108</v>
+      </c>
+      <c r="F323">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="324" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A324">
+        <v>41</v>
+      </c>
+      <c r="B324" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C324" t="s">
+        <v>623</v>
+      </c>
+      <c r="D324" t="s">
+        <v>624</v>
+      </c>
+      <c r="E324" t="s">
+        <v>108</v>
+      </c>
+      <c r="F324">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="325" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A325">
+        <v>42</v>
+      </c>
+      <c r="B325" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C325" t="s">
+        <v>625</v>
+      </c>
+      <c r="D325" t="s">
+        <v>626</v>
+      </c>
+      <c r="E325" t="s">
+        <v>108</v>
+      </c>
+      <c r="F325">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="326" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A326">
+        <v>43</v>
+      </c>
+      <c r="B326" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C326" t="s">
+        <v>360</v>
+      </c>
+      <c r="D326" t="s">
+        <v>361</v>
+      </c>
+      <c r="E326" t="s">
+        <v>627</v>
+      </c>
+      <c r="F326"/>
+    </row>
+    <row r="327" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A327">
+        <v>44</v>
+      </c>
+      <c r="B327" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C327" t="s">
+        <v>628</v>
+      </c>
+      <c r="D327" t="s">
+        <v>629</v>
+      </c>
+      <c r="E327" t="s">
+        <v>528</v>
+      </c>
+      <c r="F327"/>
+    </row>
+    <row r="328" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A328">
+        <v>45</v>
+      </c>
+      <c r="B328" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C328" t="s">
+        <v>366</v>
+      </c>
+      <c r="D328" t="s">
+        <v>367</v>
+      </c>
+      <c r="E328" t="s">
+        <v>627</v>
+      </c>
+      <c r="F328"/>
+    </row>
+    <row r="329" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A329">
+        <v>46</v>
+      </c>
+      <c r="B329" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C329" t="s">
+        <v>630</v>
+      </c>
+      <c r="D329" t="s">
+        <v>631</v>
+      </c>
+      <c r="E329" t="s">
+        <v>528</v>
+      </c>
+      <c r="F329"/>
+    </row>
+    <row r="330" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A330">
+        <v>47</v>
+      </c>
+      <c r="B330" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C330" t="s">
+        <v>632</v>
+      </c>
+      <c r="D330" t="s">
+        <v>633</v>
+      </c>
+      <c r="E330" t="s">
+        <v>528</v>
+      </c>
+      <c r="F330"/>
+    </row>
+    <row r="331" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A331">
+        <v>48</v>
+      </c>
+      <c r="B331" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C331" t="s">
+        <v>634</v>
+      </c>
+      <c r="D331" t="s">
+        <v>635</v>
+      </c>
+      <c r="E331" t="s">
+        <v>108</v>
+      </c>
+      <c r="F331">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="332" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A332">
+        <v>49</v>
+      </c>
+      <c r="B332" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C332" t="s">
+        <v>636</v>
+      </c>
+      <c r="D332" t="s">
+        <v>637</v>
+      </c>
+      <c r="E332" t="s">
+        <v>108</v>
+      </c>
+      <c r="F332">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="333" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A333">
+        <v>51</v>
+      </c>
+      <c r="B333" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C333" t="s">
+        <v>572</v>
+      </c>
+      <c r="D333" t="s">
+        <v>638</v>
+      </c>
+      <c r="E333" t="s">
+        <v>544</v>
+      </c>
+      <c r="F333"/>
+    </row>
+    <row r="334" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A334">
+        <v>52</v>
+      </c>
+      <c r="B334" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C334" t="s">
+        <v>574</v>
+      </c>
+      <c r="D334" t="s">
+        <v>639</v>
+      </c>
+      <c r="E334" t="s">
+        <v>544</v>
+      </c>
+      <c r="F334"/>
+    </row>
+    <row r="335" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A335">
+        <v>70</v>
+      </c>
+      <c r="B335" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C335" t="s">
+        <v>372</v>
+      </c>
+      <c r="D335" t="s">
+        <v>560</v>
+      </c>
+      <c r="E335" t="s">
+        <v>544</v>
+      </c>
+      <c r="F335"/>
+    </row>
+    <row r="336" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A336">
+        <v>71</v>
+      </c>
+      <c r="B336" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C336" t="s">
+        <v>374</v>
+      </c>
+      <c r="D336" t="s">
+        <v>561</v>
+      </c>
+      <c r="E336" t="s">
+        <v>544</v>
+      </c>
+      <c r="F336"/>
+    </row>
+    <row r="337" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A337">
+        <v>72</v>
+      </c>
+      <c r="B337" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C337" t="s">
+        <v>376</v>
+      </c>
+      <c r="D337" t="s">
+        <v>640</v>
+      </c>
+      <c r="E337" t="s">
+        <v>544</v>
+      </c>
+      <c r="F337"/>
+    </row>
+    <row r="338" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A338">
+        <v>73</v>
+      </c>
+      <c r="B338" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C338" t="s">
+        <v>477</v>
+      </c>
+      <c r="D338" t="s">
+        <v>641</v>
+      </c>
+      <c r="E338" t="s">
+        <v>544</v>
+      </c>
+      <c r="F338"/>
+    </row>
+    <row r="339" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A339">
+        <v>74</v>
+      </c>
+      <c r="B339" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C339" t="s">
+        <v>494</v>
+      </c>
+      <c r="D339" t="s">
+        <v>642</v>
+      </c>
+      <c r="E339" t="s">
+        <v>544</v>
+      </c>
+      <c r="F339"/>
+    </row>
+    <row r="340" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A340">
+        <v>75</v>
+      </c>
+      <c r="B340" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C340" t="s">
+        <v>496</v>
+      </c>
+      <c r="D340" t="s">
+        <v>565</v>
+      </c>
+      <c r="E340" t="s">
+        <v>544</v>
+      </c>
+      <c r="F340"/>
+    </row>
+    <row r="341" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A341">
+        <v>76</v>
+      </c>
+      <c r="B341" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C341" t="s">
+        <v>498</v>
+      </c>
+      <c r="D341" t="s">
+        <v>643</v>
+      </c>
+      <c r="E341" t="s">
+        <v>544</v>
+      </c>
+      <c r="F341"/>
+    </row>
+    <row r="342" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A342">
+        <v>77</v>
+      </c>
+      <c r="B342" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C342" t="s">
+        <v>504</v>
+      </c>
+      <c r="D342" s="15" t="s">
+        <v>567</v>
+      </c>
+      <c r="E342" t="s">
+        <v>544</v>
+      </c>
+      <c r="F342"/>
+    </row>
+    <row r="343" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A343">
+        <v>78</v>
+      </c>
+      <c r="B343" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C343" t="s">
+        <v>502</v>
+      </c>
+      <c r="D343" s="15" t="s">
+        <v>568</v>
+      </c>
+      <c r="E343" t="s">
+        <v>544</v>
+      </c>
+      <c r="F343"/>
+    </row>
+    <row r="344" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A344">
+        <v>79</v>
+      </c>
+      <c r="B344" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C344" t="s">
+        <v>500</v>
+      </c>
+      <c r="D344" t="s">
+        <v>569</v>
+      </c>
+      <c r="E344" t="s">
+        <v>544</v>
+      </c>
+      <c r="F344"/>
+    </row>
+    <row r="345" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A345">
+        <v>83</v>
+      </c>
+      <c r="B345" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C345" t="s">
+        <v>219</v>
+      </c>
+      <c r="D345" t="s">
+        <v>220</v>
+      </c>
+      <c r="E345" t="s">
+        <v>627</v>
+      </c>
+      <c r="F345"/>
+    </row>
+    <row r="346" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A346">
+        <v>84</v>
+      </c>
+      <c r="B346" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C346" t="s">
+        <v>221</v>
+      </c>
+      <c r="D346" t="s">
+        <v>222</v>
+      </c>
+      <c r="E346" t="s">
+        <v>627</v>
+      </c>
+      <c r="F346"/>
+    </row>
+    <row r="347" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A347">
+        <v>85</v>
+      </c>
+      <c r="B347" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C347" t="s">
+        <v>230</v>
+      </c>
+      <c r="D347" t="s">
+        <v>577</v>
+      </c>
+      <c r="E347" t="s">
+        <v>528</v>
+      </c>
+      <c r="F347"/>
+    </row>
+    <row r="348" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A348">
+        <v>86</v>
+      </c>
+      <c r="B348" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C348" t="s">
+        <v>328</v>
+      </c>
+      <c r="D348" t="s">
+        <v>644</v>
+      </c>
+      <c r="E348" t="s">
+        <v>108</v>
+      </c>
+      <c r="F348">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="349" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A349">
+        <v>87</v>
+      </c>
+      <c r="B349" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C349" t="s">
+        <v>326</v>
+      </c>
+      <c r="D349" t="s">
+        <v>645</v>
+      </c>
+      <c r="E349" t="s">
+        <v>108</v>
+      </c>
+      <c r="F349">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="350" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A350">
+        <v>88</v>
+      </c>
+      <c r="B350" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="C350" t="s">
+        <v>202</v>
+      </c>
+      <c r="D350" t="s">
+        <v>181</v>
+      </c>
+      <c r="E350" t="s">
+        <v>108</v>
+      </c>
+      <c r="F350">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="351" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A351">
+        <v>1</v>
+      </c>
+      <c r="B351" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C351" t="s">
+        <v>51</v>
+      </c>
+      <c r="D351" t="s">
+        <v>82</v>
+      </c>
+      <c r="E351" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="352" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A352">
+        <v>2</v>
+      </c>
+      <c r="B352" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C352" t="s">
+        <v>402</v>
+      </c>
+      <c r="D352" t="s">
+        <v>403</v>
+      </c>
+      <c r="E352" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A353">
+        <v>3</v>
+      </c>
+      <c r="B353" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C353" t="s">
+        <v>52</v>
+      </c>
+      <c r="D353" t="s">
+        <v>83</v>
+      </c>
+      <c r="E353" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A354">
+        <v>4</v>
+      </c>
+      <c r="B354" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C354" t="s">
+        <v>411</v>
+      </c>
+      <c r="D354" t="s">
+        <v>412</v>
+      </c>
+      <c r="E354" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A355">
+        <v>5</v>
+      </c>
+      <c r="B355" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C355" t="s">
+        <v>55</v>
+      </c>
+      <c r="D355" t="s">
+        <v>89</v>
+      </c>
+      <c r="E355" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A356">
+        <v>6</v>
+      </c>
+      <c r="B356" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C356" t="s">
+        <v>413</v>
+      </c>
+      <c r="D356" t="s">
+        <v>414</v>
+      </c>
+      <c r="E356" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A357">
+        <v>7</v>
+      </c>
+      <c r="B357" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C357" t="s">
+        <v>64</v>
+      </c>
+      <c r="D357" t="s">
+        <v>97</v>
+      </c>
+      <c r="E357" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A358">
+        <v>8</v>
+      </c>
+      <c r="B358" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C358" t="s">
+        <v>415</v>
+      </c>
+      <c r="D358" t="s">
+        <v>416</v>
+      </c>
+      <c r="E358" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A359">
+        <v>9</v>
+      </c>
+      <c r="B359" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C359" t="s">
+        <v>384</v>
+      </c>
+      <c r="D359" t="s">
+        <v>385</v>
+      </c>
+      <c r="E359" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A360">
+        <v>10</v>
+      </c>
+      <c r="B360" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C360" t="s">
+        <v>71</v>
+      </c>
+      <c r="D360" t="s">
+        <v>103</v>
+      </c>
+      <c r="E360" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A361">
+        <v>11</v>
+      </c>
+      <c r="B361" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C361" t="s">
+        <v>518</v>
+      </c>
+      <c r="D361" t="s">
+        <v>598</v>
+      </c>
+      <c r="E361" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A362">
+        <v>12</v>
+      </c>
+      <c r="B362" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C362" t="s">
+        <v>70</v>
+      </c>
+      <c r="D362" t="s">
+        <v>102</v>
+      </c>
+      <c r="E362" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A363">
+        <v>13</v>
+      </c>
+      <c r="B363" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C363" t="s">
+        <v>206</v>
+      </c>
+      <c r="D363" t="s">
+        <v>207</v>
+      </c>
+      <c r="E363" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A364">
+        <v>14</v>
+      </c>
+      <c r="B364" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C364" t="s">
+        <v>599</v>
+      </c>
+      <c r="D364" t="s">
+        <v>600</v>
+      </c>
+      <c r="E364" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A365">
+        <v>15</v>
+      </c>
+      <c r="B365" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C365" t="s">
+        <v>208</v>
+      </c>
+      <c r="D365" t="s">
+        <v>209</v>
+      </c>
+      <c r="E365" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A366">
+        <v>16</v>
+      </c>
+      <c r="B366" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C366" t="s">
+        <v>601</v>
+      </c>
+      <c r="D366" t="s">
+        <v>602</v>
+      </c>
+      <c r="E366" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A367">
+        <v>18</v>
+      </c>
+      <c r="B367" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C367" t="s">
+        <v>65</v>
+      </c>
+      <c r="D367" t="s">
+        <v>98</v>
+      </c>
+      <c r="E367" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A368">
+        <v>21</v>
+      </c>
+      <c r="B368" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C368" t="s">
+        <v>67</v>
+      </c>
+      <c r="D368" t="s">
+        <v>100</v>
+      </c>
+      <c r="E368" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="369" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A369">
+        <v>22</v>
+      </c>
+      <c r="B369" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C369" t="s">
+        <v>480</v>
+      </c>
+      <c r="D369" t="s">
+        <v>481</v>
+      </c>
+      <c r="E369" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="370" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A370">
+        <v>23</v>
+      </c>
+      <c r="B370" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C370" t="s">
+        <v>68</v>
+      </c>
+      <c r="D370" t="s">
+        <v>101</v>
+      </c>
+      <c r="E370" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="371" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A371">
+        <v>24</v>
+      </c>
+      <c r="B371" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C371" t="s">
+        <v>482</v>
+      </c>
+      <c r="D371" t="s">
+        <v>483</v>
+      </c>
+      <c r="E371" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="372" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A372">
+        <v>25</v>
+      </c>
+      <c r="B372" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C372" t="s">
+        <v>69</v>
+      </c>
+      <c r="D372" t="s">
+        <v>531</v>
+      </c>
+      <c r="E372" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="373" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A373">
+        <v>26</v>
+      </c>
+      <c r="B373" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C373" t="s">
+        <v>532</v>
+      </c>
+      <c r="D373" t="s">
+        <v>533</v>
+      </c>
+      <c r="E373" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="374" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A374">
+        <v>27</v>
+      </c>
+      <c r="B374" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C374" t="s">
+        <v>256</v>
+      </c>
+      <c r="D374" t="s">
+        <v>257</v>
+      </c>
+      <c r="E374" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="375" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A375">
+        <v>28</v>
+      </c>
+      <c r="B375" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C375" t="s">
+        <v>252</v>
+      </c>
+      <c r="D375" t="s">
+        <v>253</v>
+      </c>
+      <c r="E375" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="376" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A376">
+        <v>29</v>
+      </c>
+      <c r="B376" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C376" t="s">
+        <v>254</v>
+      </c>
+      <c r="D376" t="s">
+        <v>578</v>
+      </c>
+      <c r="E376" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="377" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A377">
+        <v>30</v>
+      </c>
+      <c r="B377" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C377" t="s">
+        <v>258</v>
+      </c>
+      <c r="D377" t="s">
+        <v>259</v>
+      </c>
+      <c r="E377" t="s">
+        <v>194</v>
+      </c>
+      <c r="F377">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="378" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A378">
+        <v>30</v>
+      </c>
+      <c r="B378" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C378" t="s">
+        <v>270</v>
+      </c>
+      <c r="D378" t="s">
+        <v>271</v>
+      </c>
+      <c r="E378" t="s">
+        <v>108</v>
+      </c>
+      <c r="F378">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="379" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A379">
+        <v>30</v>
+      </c>
+      <c r="B379" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C379" t="s">
+        <v>292</v>
+      </c>
+      <c r="D379" t="s">
+        <v>293</v>
+      </c>
+      <c r="E379" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="380" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A380">
+        <v>31</v>
+      </c>
+      <c r="B380" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C380" t="s">
+        <v>290</v>
+      </c>
+      <c r="D380" t="s">
+        <v>291</v>
+      </c>
+      <c r="E380" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="381" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A381">
+        <v>32</v>
+      </c>
+      <c r="B381" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C381" t="s">
+        <v>312</v>
+      </c>
+      <c r="D381" t="s">
+        <v>313</v>
+      </c>
+      <c r="E381" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="382" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A382">
+        <v>33</v>
+      </c>
+      <c r="B382" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C382" t="s">
+        <v>603</v>
+      </c>
+      <c r="D382" t="s">
+        <v>604</v>
+      </c>
+      <c r="E382" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="383" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A383">
+        <v>35</v>
+      </c>
+      <c r="B383" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C383" t="s">
+        <v>314</v>
+      </c>
+      <c r="D383" t="s">
+        <v>315</v>
+      </c>
+      <c r="E383" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="384" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A384">
+        <v>36</v>
+      </c>
+      <c r="B384" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C384" t="s">
+        <v>318</v>
+      </c>
+      <c r="D384" t="s">
+        <v>319</v>
+      </c>
+      <c r="E384" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="385" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A385">
+        <v>37</v>
+      </c>
+      <c r="B385" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C385" t="s">
+        <v>320</v>
+      </c>
+      <c r="D385" t="s">
+        <v>321</v>
+      </c>
+      <c r="E385" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="386" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A386">
+        <v>38</v>
+      </c>
+      <c r="B386" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C386" t="s">
+        <v>647</v>
+      </c>
+      <c r="D386" t="s">
+        <v>648</v>
+      </c>
+      <c r="E386" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="387" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A387">
+        <v>39</v>
+      </c>
+      <c r="B387" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C387" t="s">
+        <v>649</v>
+      </c>
+      <c r="D387" t="s">
+        <v>650</v>
+      </c>
+      <c r="E387" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="388" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A388">
+        <v>40</v>
+      </c>
+      <c r="B388" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C388" t="s">
+        <v>651</v>
+      </c>
+      <c r="D388" t="s">
+        <v>652</v>
+      </c>
+      <c r="E388" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="389" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A389">
+        <v>41</v>
+      </c>
+      <c r="B389" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C389" t="s">
+        <v>653</v>
+      </c>
+      <c r="D389" t="s">
+        <v>654</v>
+      </c>
+      <c r="E389" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="390" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A390">
+        <v>42</v>
+      </c>
+      <c r="B390" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C390" t="s">
+        <v>300</v>
+      </c>
+      <c r="D390" t="s">
+        <v>301</v>
+      </c>
+      <c r="E390" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="391" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A391">
+        <v>43</v>
+      </c>
+      <c r="B391" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C391" t="s">
+        <v>308</v>
+      </c>
+      <c r="D391" t="s">
+        <v>309</v>
+      </c>
+      <c r="E391" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="392" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A392">
+        <v>45</v>
+      </c>
+      <c r="B392" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C392" t="s">
+        <v>316</v>
+      </c>
+      <c r="D392" t="s">
+        <v>317</v>
+      </c>
+      <c r="E392" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="393" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A393">
+        <v>46</v>
+      </c>
+      <c r="B393" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C393" t="s">
+        <v>572</v>
+      </c>
+      <c r="D393" t="s">
+        <v>638</v>
+      </c>
+      <c r="E393" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="394" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A394">
+        <v>47</v>
+      </c>
+      <c r="B394" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C394" t="s">
+        <v>574</v>
+      </c>
+      <c r="D394" t="s">
+        <v>639</v>
+      </c>
+      <c r="E394" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="395" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A395">
+        <v>65</v>
+      </c>
+      <c r="B395" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C395" t="s">
+        <v>372</v>
+      </c>
+      <c r="D395" t="s">
+        <v>560</v>
+      </c>
+      <c r="E395" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="396" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A396">
+        <v>66</v>
+      </c>
+      <c r="B396" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C396" t="s">
+        <v>374</v>
+      </c>
+      <c r="D396" t="s">
+        <v>561</v>
+      </c>
+      <c r="E396" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="397" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A397">
+        <v>67</v>
+      </c>
+      <c r="B397" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C397" t="s">
+        <v>376</v>
+      </c>
+      <c r="D397" t="s">
+        <v>640</v>
+      </c>
+      <c r="E397" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="398" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A398">
+        <v>68</v>
+      </c>
+      <c r="B398" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C398" t="s">
+        <v>477</v>
+      </c>
+      <c r="D398" t="s">
+        <v>641</v>
+      </c>
+      <c r="E398" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="399" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A399">
+        <v>69</v>
+      </c>
+      <c r="B399" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C399" t="s">
+        <v>494</v>
+      </c>
+      <c r="D399" t="s">
+        <v>642</v>
+      </c>
+      <c r="E399" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="400" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A400">
+        <v>70</v>
+      </c>
+      <c r="B400" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C400" t="s">
+        <v>496</v>
+      </c>
+      <c r="D400" t="s">
+        <v>565</v>
+      </c>
+      <c r="E400" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="401" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A401">
+        <v>71</v>
+      </c>
+      <c r="B401" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C401" t="s">
+        <v>498</v>
+      </c>
+      <c r="D401" t="s">
+        <v>643</v>
+      </c>
+      <c r="E401" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="402" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A402">
+        <v>72</v>
+      </c>
+      <c r="B402" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C402" t="s">
+        <v>504</v>
+      </c>
+      <c r="D402" s="15" t="s">
+        <v>567</v>
+      </c>
+      <c r="E402" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="403" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A403">
+        <v>73</v>
+      </c>
+      <c r="B403" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C403" t="s">
+        <v>502</v>
+      </c>
+      <c r="D403" s="15" t="s">
+        <v>568</v>
+      </c>
+      <c r="E403" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="404" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A404">
+        <v>74</v>
+      </c>
+      <c r="B404" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C404" t="s">
+        <v>500</v>
+      </c>
+      <c r="D404" t="s">
+        <v>569</v>
+      </c>
+      <c r="E404" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="405" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A405">
+        <v>78</v>
+      </c>
+      <c r="B405" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C405" t="s">
+        <v>219</v>
+      </c>
+      <c r="D405" t="s">
+        <v>220</v>
+      </c>
+      <c r="E405" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="406" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A406">
+        <v>79</v>
+      </c>
+      <c r="B406" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C406" t="s">
+        <v>221</v>
+      </c>
+      <c r="D406" t="s">
+        <v>222</v>
+      </c>
+      <c r="E406" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="407" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A407">
+        <v>80</v>
+      </c>
+      <c r="B407" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C407" t="s">
+        <v>230</v>
+      </c>
+      <c r="D407" t="s">
+        <v>577</v>
+      </c>
+      <c r="E407" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="408" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A408">
+        <v>81</v>
+      </c>
+      <c r="B408" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C408" t="s">
+        <v>328</v>
+      </c>
+      <c r="D408" t="s">
+        <v>644</v>
+      </c>
+      <c r="E408" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="409" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A409">
+        <v>82</v>
+      </c>
+      <c r="B409" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C409" t="s">
+        <v>326</v>
+      </c>
+      <c r="D409" t="s">
+        <v>655</v>
+      </c>
+      <c r="E409" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="410" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A410">
+        <v>83</v>
+      </c>
+      <c r="B410" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C410" t="s">
+        <v>593</v>
+      </c>
+      <c r="D410" t="s">
+        <v>656</v>
+      </c>
+      <c r="E410" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="411" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A411">
+        <v>84</v>
+      </c>
+      <c r="B411" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C411" t="s">
+        <v>202</v>
+      </c>
+      <c r="D411" t="s">
+        <v>181</v>
+      </c>
+      <c r="E411" t="s">
+        <v>108</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:P237" xr:uid="{00000000-0009-0000-0000-000002000000}"/>

</xml_diff>

<commit_message>
#143 add more detail for NFRLT and also add AFRLT
</commit_message>
<xml_diff>
--- a/metadata/pk_spec.xlsx
+++ b/metadata/pk_spec.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeff.dickinson\Documents\GitHub\examples\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44EBC374-5540-4E84-AE0C-AD03B9623FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF0BA675-66ED-4456-B75F-25321D2A5B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2362" uniqueCount="660">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2366" uniqueCount="660">
   <si>
     <t>Attribute</t>
   </si>
@@ -2878,7 +2878,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P415"/>
+  <dimension ref="A1:P416"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" style="28" customWidth="1"/>
@@ -11306,7 +11306,7 @@
         <v>258</v>
       </c>
       <c r="D381" t="s">
-        <v>259</v>
+        <v>424</v>
       </c>
       <c r="E381" t="s">
         <v>194</v>
@@ -11336,97 +11336,97 @@
       </c>
     </row>
     <row r="383" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A383">
+      <c r="A383" s="27">
         <v>30</v>
       </c>
       <c r="B383" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C383" t="s">
-        <v>292</v>
+        <v>260</v>
       </c>
       <c r="D383" t="s">
-        <v>293</v>
+        <v>419</v>
       </c>
       <c r="E383" t="s">
-        <v>528</v>
-      </c>
-      <c r="F383" s="15">
+        <v>404</v>
+      </c>
+      <c r="F383">
         <v>8</v>
       </c>
     </row>
     <row r="384" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A384">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B384" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C384" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D384" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E384" t="s">
-        <v>108</v>
+        <v>528</v>
       </c>
       <c r="F384" s="15">
-        <v>200</v>
+        <v>8</v>
       </c>
     </row>
     <row r="385" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A385">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B385" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C385" t="s">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="D385" t="s">
-        <v>313</v>
+        <v>291</v>
       </c>
       <c r="E385" t="s">
-        <v>544</v>
+        <v>108</v>
       </c>
       <c r="F385" s="15">
-        <v>8</v>
+        <v>200</v>
       </c>
     </row>
     <row r="386" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A386">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B386" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C386" t="s">
-        <v>602</v>
+        <v>312</v>
       </c>
       <c r="D386" t="s">
-        <v>603</v>
+        <v>313</v>
       </c>
       <c r="E386" t="s">
-        <v>108</v>
+        <v>544</v>
       </c>
       <c r="F386" s="15">
-        <v>200</v>
+        <v>8</v>
       </c>
     </row>
     <row r="387" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A387">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B387" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C387" t="s">
-        <v>314</v>
+        <v>602</v>
       </c>
       <c r="D387" t="s">
-        <v>315</v>
+        <v>603</v>
       </c>
       <c r="E387" t="s">
         <v>108</v>
@@ -11437,36 +11437,36 @@
     </row>
     <row r="388" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A388">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B388" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C388" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="D388" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="E388" t="s">
-        <v>544</v>
+        <v>108</v>
       </c>
       <c r="F388" s="15">
-        <v>8</v>
+        <v>200</v>
       </c>
     </row>
     <row r="389" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A389">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B389" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C389" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D389" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="E389" t="s">
         <v>544</v>
@@ -11477,16 +11477,16 @@
     </row>
     <row r="390" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A390">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B390" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C390" t="s">
-        <v>645</v>
+        <v>320</v>
       </c>
       <c r="D390" t="s">
-        <v>646</v>
+        <v>321</v>
       </c>
       <c r="E390" t="s">
         <v>544</v>
@@ -11497,16 +11497,16 @@
     </row>
     <row r="391" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A391">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B391" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C391" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="D391" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="E391" t="s">
         <v>544</v>
@@ -11517,16 +11517,16 @@
     </row>
     <row r="392" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A392">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B392" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C392" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="D392" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="E392" t="s">
         <v>544</v>
@@ -11537,19 +11537,19 @@
     </row>
     <row r="393" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A393">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B393" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C393" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D393" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="E393" t="s">
-        <v>528</v>
+        <v>544</v>
       </c>
       <c r="F393" s="15">
         <v>8</v>
@@ -11557,19 +11557,19 @@
     </row>
     <row r="394" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A394">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B394" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C394" t="s">
-        <v>300</v>
+        <v>651</v>
       </c>
       <c r="D394" t="s">
-        <v>301</v>
+        <v>652</v>
       </c>
       <c r="E394" t="s">
-        <v>194</v>
+        <v>528</v>
       </c>
       <c r="F394" s="15">
         <v>8</v>
@@ -11580,19 +11580,19 @@
     </row>
     <row r="395" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A395">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B395" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C395" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="D395" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="E395" t="s">
-        <v>528</v>
+        <v>194</v>
       </c>
       <c r="F395" s="15">
         <v>8</v>
@@ -11600,56 +11600,56 @@
     </row>
     <row r="396" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A396">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B396" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C396" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D396" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="E396" t="s">
-        <v>108</v>
+        <v>528</v>
       </c>
       <c r="F396" s="15">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="397" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A397">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B397" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C397" t="s">
-        <v>571</v>
+        <v>316</v>
       </c>
       <c r="D397" t="s">
-        <v>636</v>
+        <v>317</v>
       </c>
       <c r="E397" t="s">
-        <v>544</v>
+        <v>108</v>
       </c>
       <c r="F397" s="15">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="398" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A398">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B398" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C398" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="D398" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="E398" t="s">
         <v>544</v>
@@ -11660,16 +11660,16 @@
     </row>
     <row r="399" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A399">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="B399" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C399" t="s">
-        <v>372</v>
+        <v>573</v>
       </c>
       <c r="D399" t="s">
-        <v>559</v>
+        <v>637</v>
       </c>
       <c r="E399" t="s">
         <v>544</v>
@@ -11680,16 +11680,16 @@
     </row>
     <row r="400" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A400">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B400" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C400" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D400" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="E400" t="s">
         <v>544</v>
@@ -11700,16 +11700,16 @@
     </row>
     <row r="401" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A401">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B401" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C401" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D401" t="s">
-        <v>638</v>
+        <v>560</v>
       </c>
       <c r="E401" t="s">
         <v>544</v>
@@ -11720,16 +11720,16 @@
     </row>
     <row r="402" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A402">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B402" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C402" t="s">
-        <v>477</v>
+        <v>376</v>
       </c>
       <c r="D402" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="E402" t="s">
         <v>544</v>
@@ -11740,16 +11740,16 @@
     </row>
     <row r="403" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A403">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B403" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C403" t="s">
-        <v>494</v>
+        <v>477</v>
       </c>
       <c r="D403" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="E403" t="s">
         <v>544</v>
@@ -11760,16 +11760,16 @@
     </row>
     <row r="404" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A404">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B404" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C404" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D404" t="s">
-        <v>564</v>
+        <v>640</v>
       </c>
       <c r="E404" t="s">
         <v>544</v>
@@ -11780,16 +11780,16 @@
     </row>
     <row r="405" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A405">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B405" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C405" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="D405" t="s">
-        <v>641</v>
+        <v>564</v>
       </c>
       <c r="E405" t="s">
         <v>544</v>
@@ -11800,16 +11800,16 @@
     </row>
     <row r="406" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A406">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B406" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C406" t="s">
-        <v>504</v>
-      </c>
-      <c r="D406" s="15" t="s">
-        <v>566</v>
+        <v>498</v>
+      </c>
+      <c r="D406" t="s">
+        <v>641</v>
       </c>
       <c r="E406" t="s">
         <v>544</v>
@@ -11820,16 +11820,16 @@
     </row>
     <row r="407" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A407">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B407" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C407" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D407" s="15" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="E407" t="s">
         <v>544</v>
@@ -11840,16 +11840,16 @@
     </row>
     <row r="408" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A408">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B408" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C408" t="s">
-        <v>500</v>
-      </c>
-      <c r="D408" t="s">
-        <v>568</v>
+        <v>502</v>
+      </c>
+      <c r="D408" s="15" t="s">
+        <v>567</v>
       </c>
       <c r="E408" t="s">
         <v>544</v>
@@ -11860,19 +11860,19 @@
     </row>
     <row r="409" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A409">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B409" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C409" t="s">
-        <v>219</v>
+        <v>500</v>
       </c>
       <c r="D409" t="s">
-        <v>220</v>
+        <v>568</v>
       </c>
       <c r="E409" t="s">
-        <v>194</v>
+        <v>544</v>
       </c>
       <c r="F409" s="15">
         <v>8</v>
@@ -11883,16 +11883,16 @@
     </row>
     <row r="410" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A410">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B410" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C410" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D410" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E410" t="s">
         <v>194</v>
@@ -11906,19 +11906,19 @@
     </row>
     <row r="411" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A411">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B411" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C411" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="D411" t="s">
-        <v>576</v>
+        <v>222</v>
       </c>
       <c r="E411" t="s">
-        <v>528</v>
+        <v>194</v>
       </c>
       <c r="F411" s="15">
         <v>8</v>
@@ -11926,36 +11926,36 @@
     </row>
     <row r="412" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A412">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B412" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C412" t="s">
-        <v>328</v>
+        <v>230</v>
       </c>
       <c r="D412" t="s">
-        <v>642</v>
+        <v>576</v>
       </c>
       <c r="E412" t="s">
-        <v>108</v>
+        <v>528</v>
       </c>
       <c r="F412" s="15">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="413" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A413">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B413" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C413" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="D413" t="s">
-        <v>653</v>
+        <v>642</v>
       </c>
       <c r="E413" t="s">
         <v>108</v>
@@ -11966,16 +11966,16 @@
     </row>
     <row r="414" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A414">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B414" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C414" t="s">
-        <v>592</v>
+        <v>326</v>
       </c>
       <c r="D414" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E414" t="s">
         <v>108</v>
@@ -11986,21 +11986,41 @@
     </row>
     <row r="415" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A415">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B415" s="15" t="s">
         <v>644</v>
       </c>
       <c r="C415" t="s">
+        <v>592</v>
+      </c>
+      <c r="D415" t="s">
+        <v>654</v>
+      </c>
+      <c r="E415" t="s">
+        <v>108</v>
+      </c>
+      <c r="F415" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="416" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A416">
+        <v>84</v>
+      </c>
+      <c r="B416" s="15" t="s">
+        <v>644</v>
+      </c>
+      <c r="C416" t="s">
         <v>202</v>
       </c>
-      <c r="D415" t="s">
+      <c r="D416" t="s">
         <v>181</v>
       </c>
-      <c r="E415" t="s">
-        <v>108</v>
-      </c>
-      <c r="F415" s="15">
+      <c r="E416" t="s">
+        <v>108</v>
+      </c>
+      <c r="F416" s="15">
         <v>1</v>
       </c>
     </row>

</xml_diff>